<commit_message>
add logger & middleware
</commit_message>
<xml_diff>
--- a/example_files/Книга1.xlsx
+++ b/example_files/Книга1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GenerateDocuments_bot\example_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647C0A5A-28D0-474F-A071-BCD50A366D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5E93578-333C-42BF-9EC5-5A098536D95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13096" xr2:uid="{F464F519-D1D3-4934-B086-DF6EC55264F3}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
-  <si>
-    <t>DOC_NAME</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>NUMBER</t>
   </si>
@@ -476,100 +473,93 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5F0FE97-D06B-4673-96A5-416CFFDDF487}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="31.1328125" customWidth="1"/>
+    <col min="3" max="3" width="12.46484375" customWidth="1"/>
+    <col min="4" max="4" width="21.265625" customWidth="1"/>
     <col min="5" max="5" width="24.6640625" customWidth="1"/>
     <col min="8" max="8" width="16.3984375" customWidth="1"/>
     <col min="9" max="9" width="16.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H1" t="s">
         <v>16</v>
       </c>
-      <c r="I1" t="s">
-        <v>17</v>
-      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="G2" s="3">
+        <v>45941.475694444445</v>
       </c>
       <c r="H2" s="3">
-        <v>45941.475694444445</v>
-      </c>
-      <c r="I2" s="3">
         <v>45942</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="2">
+        <v>14</v>
+      </c>
+      <c r="G3" s="2">
         <f>DATE(2025,10,11)</f>
         <v>45941</v>
       </c>
-      <c r="I3" s="2">
+      <c r="H3" s="2">
         <f>DATE(2025,10,11)</f>
         <v>45941</v>
       </c>

</xml_diff>